<commit_message>
Corregir cardinalidades F17 y F24 del Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013aHpfjvs4B5gdaSHRxJk6F
</commit_message>
<xml_diff>
--- a/ENUNCIADO_ACTIVIDAD_BANCO_corregido.xlsx
+++ b/ENUNCIADO_ACTIVIDAD_BANCO_corregido.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -39,14 +39,6 @@
       <b val="1"/>
       <color theme="1"/>
       <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -157,18 +149,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -180,9 +171,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -582,23 +580,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col width="19.109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="15.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="20.109375" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="22.77734375" bestFit="1" customWidth="1" min="4" max="5"/>
-    <col width="18.21875" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="21.21875" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="20" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="28.6640625" customWidth="1" min="9" max="9"/>
-    <col width="17.33203125" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="19.33203125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="19.109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
+    <col width="15.44140625" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="20.109375" bestFit="1" customWidth="1" style="10" min="3" max="3"/>
+    <col width="22.77734375" bestFit="1" customWidth="1" style="10" min="4" max="5"/>
+    <col width="18.21875" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
+    <col width="21.21875" bestFit="1" customWidth="1" style="10" min="7" max="7"/>
+    <col width="20" bestFit="1" customWidth="1" style="10" min="8" max="8"/>
+    <col width="28.6640625" customWidth="1" style="10" min="9" max="9"/>
+    <col width="17.33203125" bestFit="1" customWidth="1" style="10" min="11" max="11"/>
+    <col width="19.33203125" bestFit="1" customWidth="1" style="10" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>ENTIDADES</t>
         </is>
@@ -660,8 +658,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n"/>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="11" t="n"/>
+      <c r="B2" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
@@ -717,8 +715,8 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28.8" customHeight="1">
-      <c r="A3" s="10" t="n"/>
+    <row r="3" ht="28.8" customHeight="1" s="10">
+      <c r="A3" s="11" t="n"/>
       <c r="B3" t="inlineStr">
         <is>
           <t xml:space="preserve">LOCALIDAD </t>
@@ -776,7 +774,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n"/>
+      <c r="A4" s="11" t="n"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>ACTIVOS</t>
@@ -792,7 +790,7 @@
           <t>FECHA ULTIMO ACCESO</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>SUCURSAL</t>
         </is>
@@ -809,7 +807,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n"/>
+      <c r="A5" s="11" t="n"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>CIUDAD</t>
@@ -827,7 +825,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n"/>
+      <c r="A6" s="11" t="n"/>
       <c r="C6" t="inlineStr">
         <is>
           <t xml:space="preserve">ID EMPLEADO </t>
@@ -840,10 +838,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-    </row>
-    <row r="16" ht="14.4" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A7" s="12" t="n"/>
+    </row>
+    <row r="16" ht="14.4" customHeight="1" s="10">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>RELACIONES</t>
         </is>
@@ -889,261 +887,303 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="39.6" customHeight="1">
-      <c r="B17" s="5" t="inlineStr">
+    <row r="17" ht="39.6" customHeight="1" s="10">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>asesora</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>EMPLEADO</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>1:N</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>(0,1)</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>(0,n)</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Cada cliente tiene como mucho un asesor; un empleado asesora a varios clientes.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26.4" customHeight="1">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="18" ht="26.4" customHeight="1" s="10">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>es jefe de</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>EMPLEADO</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>EMPLEADO</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>1:N</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>(0,1) jefe</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>(0,n) subordinados</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Reflexiva: el jefe también es un empleado.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="39.6" customHeight="1">
-      <c r="B19" s="5" t="inlineStr">
+    <row r="19" ht="39.6" customHeight="1" s="10">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>es titular de</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>CUENTA</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>N:M</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>(1,n)</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>(0,n)</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>fecha_ultimo_acceso</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>"Más de un titular" y "más de una cuenta". La fecha depende del cliente Y de la cuenta.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="39.6" customHeight="1">
-      <c r="B20" s="5" t="inlineStr">
+    <row r="20" ht="39.6" customHeight="1" s="10">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>es titular de</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>PRÉSTAMO</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>N:M</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>(1,n)</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>(0,n)</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Un préstamo tiene uno o más titulares; un cliente puede pedir varios préstamos.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="26.4" customHeight="1">
-      <c r="B21" s="5" t="inlineStr">
+    <row r="21" ht="26.4" customHeight="1" s="10">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>concede</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>SUCURSAL</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>PRÉSTAMO</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>1:N</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>(1,1)</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>(0,n)</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>"Cada préstamo se ofrece desde una sucursal concreta".</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26.4" customHeight="1">
-      <c r="B22" s="5" t="inlineStr">
+    <row r="22" ht="26.4" customHeight="1" s="10">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>tiene (ID)</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>PRÉSTAMO</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>PAGO</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>1:N</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>(1,1)</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>(0,n)</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Dependencia de identificación: PAGO es entidad débil.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="39.6" customHeight="1">
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="6" t="inlineStr">
+    <row r="23" ht="39.6" customHeight="1" s="10">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>tiene (ID)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>CUENTA</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>CUENTA_AHORRO / CUENTA_CORRIENTE</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>total y exclusiva</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Supuesto: toda cuenta es de ahorro O corriente, nunca las dos ni ninguna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="43.2" customHeight="1" s="10">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>tiene (ID)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>EMPLEADO</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>PERSONAS_A_CARGO</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>1:N</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>(1,1)</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>(0,n)</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Dependencia de identificación: PERSONAS_A_CARGO es entidad débil.</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1205,10 @@
   <dimension ref="A2:H17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col width="59.109375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="14.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="29.109375" bestFit="1" customWidth="1" min="5" max="6"/>
-    <col width="18.88671875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="59.109375" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="14.6640625" bestFit="1" customWidth="1" style="10" min="3" max="3"/>
+    <col width="29.109375" bestFit="1" customWidth="1" style="10" min="5" max="6"/>
+    <col width="18.88671875" bestFit="1" customWidth="1" style="10" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">

</xml_diff>